<commit_message>
Shorten Excel sheet names to Excel 31-char limit
Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/fno_contratacoes_2000_2021_ipca.xlsx
+++ b/output/fno_contratacoes_2000_2021_ipca.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Demonstrativo_reversao_IGPDI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Reversao_IGPDI" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Reversao_R$_bi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Alternativa_grafico_como_corrente" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Alternativa_R$_bi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Alt_grafico_corrente" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Alt_R$_bi" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Oficial_parcial_IPCA" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Confronto_oficial" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Metodologia" sheetId="7" state="visible" r:id="rId7"/>

</xml_diff>